<commit_message>
finished the team for iem rio groups
</commit_message>
<xml_diff>
--- a/test_multi.xlsx
+++ b/test_multi.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emilio.cornejo\Desktop\fantasy\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B07FC4D6-23EA-4DE7-86B3-846B7412B7B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6E0CE4CF-2F2E-4E6F-92D3-F6D95893AE77}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="1650" windowWidth="29040" windowHeight="15720" xr2:uid="{23D2E913-A0C1-4AB9-9120-D8F79DF3DCE7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{23D2E913-A0C1-4AB9-9120-D8F79DF3DCE7}"/>
   </bookViews>
   <sheets>
     <sheet name="multiplier" sheetId="1" r:id="rId1"/>

</xml_diff>